<commit_message>
Auto backup 2026-07-01 01:35:03
</commit_message>
<xml_diff>
--- a/SwissTechAhsan/AHSAN/carry world.xlsx
+++ b/SwissTechAhsan/AHSAN/carry world.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="20">
   <si>
     <t xml:space="preserve">DATE </t>
   </si>
@@ -81,6 +81,9 @@
   </si>
   <si>
     <t>WAQAS ABDUL WAHAB</t>
+  </si>
+  <si>
+    <t>AL WAHAB</t>
   </si>
 </sst>
 </file>
@@ -449,7 +452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:M57"/>
+  <dimension ref="A2:M58"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.21875" customWidth="1"/>
@@ -540,17 +543,15 @@
       <c r="M6" s="9"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A7" s="2">
-        <v>4</v>
-      </c>
+      <c r="A7" s="2"/>
       <c r="B7" s="5">
         <v>46177</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D7" s="4">
-        <v>118000</v>
+        <v>248000</v>
       </c>
       <c r="J7" s="7"/>
       <c r="K7" s="8"/>
@@ -559,16 +560,16 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" s="5">
-        <v>46178</v>
+        <v>46177</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D8" s="4">
-        <v>270000</v>
+        <v>118000</v>
       </c>
       <c r="J8" s="7"/>
       <c r="K8" s="8"/>
@@ -577,16 +578,16 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B9" s="5">
         <v>46178</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D9" s="4">
-        <v>200000</v>
+        <v>270000</v>
       </c>
       <c r="J9" s="7"/>
       <c r="K9" s="8"/>
@@ -595,16 +596,16 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B10" s="5">
         <v>46178</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D10" s="4">
-        <v>247000</v>
+        <v>200000</v>
       </c>
       <c r="J10" s="7"/>
       <c r="K10" s="8"/>
@@ -613,16 +614,16 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B11" s="5">
         <v>46178</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D11" s="4">
-        <v>234000</v>
+        <v>247000</v>
       </c>
       <c r="J11" s="7"/>
       <c r="K11" s="8"/>
@@ -631,16 +632,16 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5">
+        <v>46178</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="5">
-        <v>46179</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="D12" s="4">
-        <v>100000</v>
+        <v>234000</v>
       </c>
       <c r="J12" s="7"/>
       <c r="K12" s="8"/>
@@ -649,16 +650,16 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B13" s="5">
         <v>46179</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D13" s="4">
-        <v>179000</v>
+        <v>100000</v>
       </c>
       <c r="J13" s="7"/>
       <c r="K13" s="8"/>
@@ -667,16 +668,16 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B14" s="5">
         <v>46179</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D14" s="4">
-        <v>200000</v>
+        <v>179000</v>
       </c>
       <c r="J14" s="7"/>
       <c r="K14" s="8"/>
@@ -685,16 +686,16 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15" s="5">
         <v>46179</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D15" s="4">
-        <v>150000</v>
+        <v>200000</v>
       </c>
       <c r="J15" s="7"/>
       <c r="K15" s="8"/>
@@ -703,16 +704,16 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B16" s="5">
-        <v>46180</v>
+        <v>46179</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D16" s="4">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="J16" s="7"/>
       <c r="K16" s="8"/>
@@ -721,16 +722,16 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B17" s="5">
-        <v>46181</v>
+        <v>46180</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D17" s="4">
-        <v>185000</v>
+        <v>100000</v>
       </c>
       <c r="J17" s="7"/>
       <c r="K17" s="8"/>
@@ -739,16 +740,16 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B18" s="5">
         <v>46181</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D18" s="4">
-        <v>91000</v>
+        <v>185000</v>
       </c>
       <c r="J18" s="7"/>
       <c r="K18" s="8"/>
@@ -757,16 +758,16 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B19" s="5">
         <v>46181</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D19" s="4">
-        <v>150000</v>
+        <v>91000</v>
       </c>
       <c r="J19" s="7"/>
       <c r="K19" s="8"/>
@@ -775,16 +776,16 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B20" s="5">
         <v>46181</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D20" s="4">
-        <v>66000</v>
+        <v>150000</v>
       </c>
       <c r="J20" s="7"/>
       <c r="K20" s="8"/>
@@ -793,16 +794,16 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B21" s="5">
-        <v>46182</v>
+        <v>46181</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D21" s="4">
-        <v>150000</v>
+        <v>66000</v>
       </c>
       <c r="J21" s="7"/>
       <c r="K21" s="8"/>
@@ -811,13 +812,13 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B22" s="5">
-        <v>46183</v>
+        <v>46182</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D22" s="4">
         <v>150000</v>
@@ -829,19 +830,16 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B23" s="5">
         <v>46183</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D23" s="4">
         <v>150000</v>
-      </c>
-      <c r="F23" t="s">
-        <v>16</v>
       </c>
       <c r="J23" s="7"/>
       <c r="K23" s="8"/>
@@ -850,16 +848,19 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B24" s="5">
-        <v>46184</v>
+        <v>46183</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D24" s="4">
         <v>150000</v>
+      </c>
+      <c r="F24" t="s">
+        <v>16</v>
       </c>
       <c r="J24" s="7"/>
       <c r="K24" s="8"/>
@@ -868,13 +869,13 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B25" s="5">
         <v>46184</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D25" s="4">
         <v>150000</v>
@@ -886,16 +887,16 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B26" s="5">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D26" s="4">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="J26" s="7"/>
       <c r="K26" s="8"/>
@@ -904,16 +905,16 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B27" s="5">
-        <v>46186</v>
+        <v>46185</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D27" s="4">
-        <v>150000</v>
+        <v>200000</v>
       </c>
       <c r="J27" s="7"/>
       <c r="K27" s="8"/>
@@ -922,16 +923,16 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B28" s="5">
-        <v>46188</v>
+        <v>46186</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="D28" s="4">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="J28" s="7"/>
       <c r="K28" s="8"/>
@@ -940,16 +941,16 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B29" s="5">
         <v>46188</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="D29" s="4">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="J29" s="7"/>
       <c r="K29" s="8"/>
@@ -958,16 +959,16 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B30" s="5">
-        <v>46189</v>
+        <v>46188</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D30" s="4">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="J30" s="7"/>
       <c r="K30" s="8"/>
@@ -976,16 +977,16 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B31" s="5">
         <v>46189</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="D31" s="4">
-        <v>39000</v>
+        <v>100000</v>
       </c>
       <c r="J31" s="7"/>
       <c r="K31" s="8"/>
@@ -994,16 +995,16 @@
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B32" s="5">
         <v>46189</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="D32" s="4">
-        <v>150000</v>
+        <v>39000</v>
       </c>
       <c r="J32" s="7"/>
       <c r="K32" s="8"/>
@@ -1012,13 +1013,13 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B33" s="5">
-        <v>46190</v>
+        <v>46189</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D33" s="4">
         <v>150000</v>
@@ -1030,16 +1031,16 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B34" s="5">
         <v>46190</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="D34" s="4">
-        <v>50000</v>
+        <v>150000</v>
       </c>
       <c r="J34" s="7"/>
       <c r="K34" s="8"/>
@@ -1048,16 +1049,16 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B35" s="5">
-        <v>46191</v>
+        <v>46190</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="D35" s="4">
-        <v>150000</v>
+        <v>50000</v>
       </c>
       <c r="J35" s="7"/>
       <c r="K35" s="8"/>
@@ -1066,10 +1067,10 @@
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B36" s="5">
-        <v>46192</v>
+        <v>46191</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>4</v>
@@ -1078,40 +1079,40 @@
         <v>150000</v>
       </c>
       <c r="J36" s="7"/>
-      <c r="K36" s="7"/>
+      <c r="K36" s="8"/>
       <c r="L36" s="7"/>
       <c r="M36" s="9"/>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B37" s="5">
         <v>46192</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="D37" s="4">
-        <v>13000</v>
+        <v>150000</v>
       </c>
       <c r="J37" s="7"/>
       <c r="K37" s="7"/>
       <c r="L37" s="7"/>
-      <c r="M37" s="7"/>
+      <c r="M37" s="9"/>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B38" s="5">
         <v>46192</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D38" s="4">
-        <v>160000</v>
+        <v>13000</v>
       </c>
       <c r="J38" s="7"/>
       <c r="K38" s="7"/>
@@ -1120,41 +1121,45 @@
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B39" s="5">
-        <v>46193</v>
+        <v>46192</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D39" s="4">
-        <v>250000</v>
-      </c>
+        <v>160000</v>
+      </c>
+      <c r="J39" s="7"/>
+      <c r="K39" s="7"/>
+      <c r="L39" s="7"/>
+      <c r="M39" s="7"/>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B40" s="5">
         <v>46193</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D40" s="4">
-        <v>150000</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B41" s="5">
-        <v>46194</v>
+        <v>46193</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D41" s="4">
         <v>150000</v>
@@ -1162,13 +1167,13 @@
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B42" s="5">
         <v>46194</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D42" s="4">
         <v>150000</v>
@@ -1176,10 +1181,10 @@
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B43" s="5">
-        <v>46196</v>
+        <v>46194</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>4</v>
@@ -1190,128 +1195,136 @@
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B44" s="5">
-        <v>46200</v>
+        <v>46196</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D44" s="4">
-        <v>94500</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B45" s="5">
         <v>46200</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D45" s="4">
-        <v>200000</v>
+        <v>94500</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B46" s="5">
-        <v>46201</v>
+        <v>46200</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D46" s="4">
-        <v>40000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
-        <v>44</v>
-      </c>
-      <c r="B47" s="10">
-        <v>46202</v>
+        <v>43</v>
+      </c>
+      <c r="B47" s="5">
+        <v>46201</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="D47" s="4">
-        <v>257000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B48" s="10">
-        <v>46203</v>
+        <v>46202</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D48" s="4">
-        <v>150000</v>
+        <v>257000</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B49" s="10">
         <v>46203</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D49" s="4">
-        <v>100000</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B50" s="10">
         <v>46203</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="D50" s="4">
-        <v>58000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
-        <v>48</v>
-      </c>
-      <c r="B51" s="10"/>
-      <c r="C51" s="2"/>
-      <c r="D51" s="4"/>
+        <v>47</v>
+      </c>
+      <c r="B51" s="10">
+        <v>46203</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D51" s="4">
+        <v>58000</v>
+      </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
-        <v>49</v>
-      </c>
-      <c r="B52" s="2"/>
+        <v>48</v>
+      </c>
+      <c r="B52" s="10"/>
       <c r="C52" s="2"/>
       <c r="D52" s="4"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
       <c r="D53" s="4"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A54" s="2"/>
+      <c r="A54" s="2">
+        <v>50</v>
+      </c>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
       <c r="D54" s="4"/>
@@ -1334,6 +1347,12 @@
       <c r="C57" s="2"/>
       <c r="D57" s="4"/>
     </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A58" s="2"/>
+      <c r="B58" s="2"/>
+      <c r="C58" s="2"/>
+      <c r="D58" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Auto backup 2026-07-01 02:35:02
</commit_message>
<xml_diff>
--- a/SwissTechAhsan/AHSAN/carry world.xlsx
+++ b/SwissTechAhsan/AHSAN/carry world.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="22">
   <si>
     <t xml:space="preserve">DATE </t>
   </si>
@@ -84,6 +84,12 @@
   </si>
   <si>
     <t>AL WAHAB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A- WAHAB </t>
+  </si>
+  <si>
+    <t>Z.U ONLIME</t>
   </si>
 </sst>
 </file>
@@ -452,7 +458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:M58"/>
+  <dimension ref="A2:M60"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.21875" customWidth="1"/>
@@ -811,17 +817,15 @@
       <c r="M21" s="9"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A22" s="2">
-        <v>18</v>
-      </c>
+      <c r="A22" s="2"/>
       <c r="B22" s="5">
         <v>46182</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="D22" s="4">
-        <v>150000</v>
+        <v>194000</v>
       </c>
       <c r="J22" s="7"/>
       <c r="K22" s="8"/>
@@ -830,13 +834,13 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B23" s="5">
-        <v>46183</v>
+        <v>46182</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D23" s="4">
         <v>150000</v>
@@ -848,19 +852,16 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B24" s="5">
         <v>46183</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D24" s="4">
         <v>150000</v>
-      </c>
-      <c r="F24" t="s">
-        <v>16</v>
       </c>
       <c r="J24" s="7"/>
       <c r="K24" s="8"/>
@@ -869,16 +870,19 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B25" s="5">
-        <v>46184</v>
+        <v>46183</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D25" s="4">
         <v>150000</v>
+      </c>
+      <c r="F25" t="s">
+        <v>16</v>
       </c>
       <c r="J25" s="7"/>
       <c r="K25" s="8"/>
@@ -886,17 +890,15 @@
       <c r="M25" s="9"/>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A26" s="2">
-        <v>22</v>
-      </c>
+      <c r="A26" s="2"/>
       <c r="B26" s="5">
         <v>46184</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="D26" s="4">
-        <v>150000</v>
+        <v>273000</v>
       </c>
       <c r="J26" s="7"/>
       <c r="K26" s="8"/>
@@ -905,16 +907,16 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B27" s="5">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D27" s="4">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="J27" s="7"/>
       <c r="K27" s="8"/>
@@ -923,10 +925,10 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B28" s="5">
-        <v>46186</v>
+        <v>46184</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>4</v>
@@ -941,16 +943,16 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B29" s="5">
-        <v>46188</v>
+        <v>46185</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="D29" s="4">
-        <v>100000</v>
+        <v>200000</v>
       </c>
       <c r="J29" s="7"/>
       <c r="K29" s="8"/>
@@ -959,10 +961,10 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B30" s="5">
-        <v>46188</v>
+        <v>46186</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>4</v>
@@ -977,13 +979,13 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B31" s="5">
-        <v>46189</v>
+        <v>46188</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D31" s="4">
         <v>100000</v>
@@ -995,16 +997,16 @@
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B32" s="5">
-        <v>46189</v>
+        <v>46188</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="D32" s="4">
-        <v>39000</v>
+        <v>150000</v>
       </c>
       <c r="J32" s="7"/>
       <c r="K32" s="8"/>
@@ -1013,16 +1015,16 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B33" s="5">
         <v>46189</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D33" s="4">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="J33" s="7"/>
       <c r="K33" s="8"/>
@@ -1031,16 +1033,16 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B34" s="5">
-        <v>46190</v>
+        <v>46189</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D34" s="4">
-        <v>150000</v>
+        <v>39000</v>
       </c>
       <c r="J34" s="7"/>
       <c r="K34" s="8"/>
@@ -1049,16 +1051,16 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B35" s="5">
-        <v>46190</v>
+        <v>46189</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="D35" s="4">
-        <v>50000</v>
+        <v>150000</v>
       </c>
       <c r="J35" s="7"/>
       <c r="K35" s="8"/>
@@ -1067,13 +1069,13 @@
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B36" s="5">
-        <v>46191</v>
+        <v>46190</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D36" s="4">
         <v>150000</v>
@@ -1085,106 +1087,114 @@
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B37" s="5">
-        <v>46192</v>
+        <v>46190</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="D37" s="4">
-        <v>150000</v>
+        <v>50000</v>
       </c>
       <c r="J37" s="7"/>
-      <c r="K37" s="7"/>
+      <c r="K37" s="8"/>
       <c r="L37" s="7"/>
       <c r="M37" s="9"/>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B38" s="5">
-        <v>46192</v>
+        <v>46191</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="D38" s="4">
-        <v>13000</v>
+        <v>150000</v>
       </c>
       <c r="J38" s="7"/>
-      <c r="K38" s="7"/>
+      <c r="K38" s="8"/>
       <c r="L38" s="7"/>
-      <c r="M38" s="7"/>
+      <c r="M38" s="9"/>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B39" s="5">
         <v>46192</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="D39" s="4">
-        <v>160000</v>
+        <v>150000</v>
       </c>
       <c r="J39" s="7"/>
       <c r="K39" s="7"/>
       <c r="L39" s="7"/>
-      <c r="M39" s="7"/>
+      <c r="M39" s="9"/>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B40" s="5">
-        <v>46193</v>
+        <v>46192</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D40" s="4">
-        <v>250000</v>
-      </c>
+        <v>13000</v>
+      </c>
+      <c r="J40" s="7"/>
+      <c r="K40" s="7"/>
+      <c r="L40" s="7"/>
+      <c r="M40" s="7"/>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B41" s="5">
-        <v>46193</v>
+        <v>46192</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="D41" s="4">
-        <v>150000</v>
-      </c>
+        <v>160000</v>
+      </c>
+      <c r="J41" s="7"/>
+      <c r="K41" s="7"/>
+      <c r="L41" s="7"/>
+      <c r="M41" s="7"/>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B42" s="5">
-        <v>46194</v>
+        <v>46193</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D42" s="4">
-        <v>150000</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B43" s="5">
-        <v>46194</v>
+        <v>46193</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>4</v>
@@ -1195,13 +1205,13 @@
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B44" s="5">
-        <v>46196</v>
+        <v>46194</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D44" s="4">
         <v>150000</v>
@@ -1209,134 +1219,150 @@
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B45" s="5">
-        <v>46200</v>
+        <v>46194</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D45" s="4">
-        <v>94500</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B46" s="5">
-        <v>46200</v>
+        <v>46196</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D46" s="4">
-        <v>200000</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B47" s="5">
-        <v>46201</v>
+        <v>46200</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D47" s="4">
-        <v>40000</v>
+        <v>94500</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
-        <v>44</v>
-      </c>
-      <c r="B48" s="10">
-        <v>46202</v>
+        <v>42</v>
+      </c>
+      <c r="B48" s="5">
+        <v>46200</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="D48" s="4">
-        <v>257000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
-        <v>45</v>
-      </c>
-      <c r="B49" s="10">
-        <v>46203</v>
+        <v>43</v>
+      </c>
+      <c r="B49" s="5">
+        <v>46201</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D49" s="4">
-        <v>150000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B50" s="10">
-        <v>46203</v>
+        <v>46202</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="D50" s="4">
-        <v>100000</v>
+        <v>257000</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B51" s="10">
         <v>46203</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D51" s="4">
-        <v>58000</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
-        <v>48</v>
-      </c>
-      <c r="B52" s="10"/>
-      <c r="C52" s="2"/>
-      <c r="D52" s="4"/>
+        <v>46</v>
+      </c>
+      <c r="B52" s="10">
+        <v>46203</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D52" s="4">
+        <v>100000</v>
+      </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
-        <v>49</v>
-      </c>
-      <c r="B53" s="2"/>
-      <c r="C53" s="2"/>
-      <c r="D53" s="4"/>
+        <v>47</v>
+      </c>
+      <c r="B53" s="10">
+        <v>46203</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D53" s="4">
+        <v>58000</v>
+      </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
-        <v>50</v>
-      </c>
-      <c r="B54" s="2"/>
+        <v>48</v>
+      </c>
+      <c r="B54" s="10"/>
       <c r="C54" s="2"/>
       <c r="D54" s="4"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A55" s="2"/>
+      <c r="A55" s="2">
+        <v>49</v>
+      </c>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
       <c r="D55" s="4"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A56" s="2"/>
+      <c r="A56" s="2">
+        <v>50</v>
+      </c>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
       <c r="D56" s="4"/>
@@ -1353,6 +1379,18 @@
       <c r="C58" s="2"/>
       <c r="D58" s="4"/>
     </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A59" s="2"/>
+      <c r="B59" s="2"/>
+      <c r="C59" s="2"/>
+      <c r="D59" s="4"/>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A60" s="2"/>
+      <c r="B60" s="2"/>
+      <c r="C60" s="2"/>
+      <c r="D60" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Auto backup 2026-07-01 08:05:02
</commit_message>
<xml_diff>
--- a/SwissTechAhsan/AHSAN/carry world.xlsx
+++ b/SwissTechAhsan/AHSAN/carry world.xlsx
@@ -9,10 +9,11 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="14304"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="14304" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="carry world june 2026" sheetId="1" r:id="rId1"/>
+    <sheet name="carry world july2026" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="22">
   <si>
     <t xml:space="preserve">DATE </t>
   </si>
@@ -1395,4 +1396,464 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.5546875" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" customWidth="1"/>
+    <col min="3" max="3" width="30.44140625" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="5">
+        <v>46204</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="4">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
+        <v>2</v>
+      </c>
+      <c r="B4" s="5"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
+        <v>3</v>
+      </c>
+      <c r="B5" s="5"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="2"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="4"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
+        <v>4</v>
+      </c>
+      <c r="B7" s="5"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="2">
+        <v>5</v>
+      </c>
+      <c r="B8" s="5"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="4"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="2">
+        <v>6</v>
+      </c>
+      <c r="B9" s="5"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="2">
+        <v>7</v>
+      </c>
+      <c r="B10" s="5"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="4"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="2">
+        <v>8</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="4"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="2">
+        <v>9</v>
+      </c>
+      <c r="B12" s="5"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="4"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="2">
+        <v>10</v>
+      </c>
+      <c r="B13" s="5"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="4"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="2">
+        <v>11</v>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="4"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="2">
+        <v>12</v>
+      </c>
+      <c r="B15" s="5"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="4"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="2">
+        <v>13</v>
+      </c>
+      <c r="B16" s="5"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="4"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="2">
+        <v>14</v>
+      </c>
+      <c r="B17" s="5"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="4"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="2">
+        <v>15</v>
+      </c>
+      <c r="B18" s="5"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="4"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="2">
+        <v>16</v>
+      </c>
+      <c r="B19" s="5"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="4"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="2">
+        <v>17</v>
+      </c>
+      <c r="B20" s="5"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="4"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="2"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="4"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="2">
+        <v>18</v>
+      </c>
+      <c r="B22" s="5"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="4"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="2">
+        <v>19</v>
+      </c>
+      <c r="B23" s="5"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="4"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="2">
+        <v>20</v>
+      </c>
+      <c r="B24" s="5"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="4"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="2"/>
+      <c r="B25" s="5"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="4"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="2">
+        <v>21</v>
+      </c>
+      <c r="B26" s="5"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="4"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="2">
+        <v>22</v>
+      </c>
+      <c r="B27" s="5"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="4"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="2">
+        <v>23</v>
+      </c>
+      <c r="B28" s="5"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="4"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="2">
+        <v>24</v>
+      </c>
+      <c r="B29" s="5"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="4"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="2">
+        <v>25</v>
+      </c>
+      <c r="B30" s="5"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="4"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="2">
+        <v>26</v>
+      </c>
+      <c r="B31" s="5"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="4"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="2">
+        <v>27</v>
+      </c>
+      <c r="B32" s="5"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="4"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="2">
+        <v>28</v>
+      </c>
+      <c r="B33" s="5"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="4"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="2">
+        <v>29</v>
+      </c>
+      <c r="B34" s="5"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="4"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="2">
+        <v>30</v>
+      </c>
+      <c r="B35" s="5"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="4"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="2">
+        <v>31</v>
+      </c>
+      <c r="B36" s="5"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="4"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="2">
+        <v>32</v>
+      </c>
+      <c r="B37" s="5"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="4"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" s="2">
+        <v>33</v>
+      </c>
+      <c r="B38" s="5"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="4"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" s="2">
+        <v>34</v>
+      </c>
+      <c r="B39" s="5"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="4"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" s="2">
+        <v>35</v>
+      </c>
+      <c r="B40" s="5"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="4"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" s="2">
+        <v>36</v>
+      </c>
+      <c r="B41" s="5"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="4"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" s="2">
+        <v>37</v>
+      </c>
+      <c r="B42" s="5"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="4"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" s="2">
+        <v>38</v>
+      </c>
+      <c r="B43" s="5"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="4"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" s="2">
+        <v>39</v>
+      </c>
+      <c r="B44" s="5"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="4"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" s="2">
+        <v>40</v>
+      </c>
+      <c r="B45" s="5"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="4"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A46" s="2">
+        <v>41</v>
+      </c>
+      <c r="B46" s="5"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="4"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" s="2">
+        <v>42</v>
+      </c>
+      <c r="B47" s="5"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="4"/>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" s="2">
+        <v>43</v>
+      </c>
+      <c r="B48" s="5"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="4"/>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" s="2">
+        <v>44</v>
+      </c>
+      <c r="B49" s="10"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="4"/>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" s="2">
+        <v>45</v>
+      </c>
+      <c r="B50" s="10"/>
+      <c r="C50" s="2"/>
+      <c r="D50" s="4"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" s="2">
+        <v>46</v>
+      </c>
+      <c r="B51" s="10"/>
+      <c r="C51" s="2"/>
+      <c r="D51" s="4"/>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" s="2">
+        <v>47</v>
+      </c>
+      <c r="B52" s="10"/>
+      <c r="C52" s="2"/>
+      <c r="D52" s="4"/>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A53" s="2">
+        <v>48</v>
+      </c>
+      <c r="B53" s="10"/>
+      <c r="C53" s="2"/>
+      <c r="D53" s="4"/>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" s="2">
+        <v>49</v>
+      </c>
+      <c r="B54" s="2"/>
+      <c r="C54" s="2"/>
+      <c r="D54" s="4"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" s="2">
+        <v>50</v>
+      </c>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Auto backup 2026-07-01 11:05:02
</commit_message>
<xml_diff>
--- a/SwissTechAhsan/AHSAN/carry world.xlsx
+++ b/SwissTechAhsan/AHSAN/carry world.xlsx
@@ -550,7 +550,9 @@
       <c r="M6" s="9"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A7" s="2"/>
+      <c r="A7" s="2">
+        <v>4</v>
+      </c>
       <c r="B7" s="5">
         <v>46177</v>
       </c>
@@ -567,7 +569,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B8" s="5">
         <v>46177</v>
@@ -585,7 +587,7 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B9" s="5">
         <v>46178</v>
@@ -603,7 +605,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B10" s="5">
         <v>46178</v>
@@ -621,7 +623,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B11" s="5">
         <v>46178</v>
@@ -639,7 +641,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B12" s="5">
         <v>46178</v>
@@ -657,7 +659,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B13" s="5">
         <v>46179</v>
@@ -675,7 +677,7 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B14" s="5">
         <v>46179</v>
@@ -693,7 +695,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B15" s="5">
         <v>46179</v>
@@ -711,7 +713,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B16" s="5">
         <v>46179</v>
@@ -729,7 +731,7 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B17" s="5">
         <v>46180</v>
@@ -747,7 +749,7 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B18" s="5">
         <v>46181</v>
@@ -765,7 +767,7 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B19" s="5">
         <v>46181</v>
@@ -783,7 +785,7 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B20" s="5">
         <v>46181</v>
@@ -801,7 +803,7 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B21" s="5">
         <v>46181</v>
@@ -818,7 +820,9 @@
       <c r="M21" s="9"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A22" s="2"/>
+      <c r="A22" s="2">
+        <v>19</v>
+      </c>
       <c r="B22" s="5">
         <v>46182</v>
       </c>
@@ -835,7 +839,7 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B23" s="5">
         <v>46182</v>
@@ -853,7 +857,7 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B24" s="5">
         <v>46183</v>
@@ -871,7 +875,7 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B25" s="5">
         <v>46183</v>
@@ -891,7 +895,9 @@
       <c r="M25" s="9"/>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A26" s="2"/>
+      <c r="A26" s="2">
+        <v>23</v>
+      </c>
       <c r="B26" s="5">
         <v>46184</v>
       </c>
@@ -908,7 +914,7 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B27" s="5">
         <v>46184</v>
@@ -926,7 +932,7 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B28" s="5">
         <v>46184</v>
@@ -944,7 +950,7 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B29" s="5">
         <v>46185</v>
@@ -962,7 +968,7 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B30" s="5">
         <v>46186</v>
@@ -980,7 +986,7 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B31" s="5">
         <v>46188</v>
@@ -998,7 +1004,7 @@
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B32" s="5">
         <v>46188</v>
@@ -1016,7 +1022,7 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B33" s="5">
         <v>46189</v>
@@ -1034,7 +1040,7 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B34" s="5">
         <v>46189</v>
@@ -1052,7 +1058,7 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B35" s="5">
         <v>46189</v>
@@ -1070,7 +1076,7 @@
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B36" s="5">
         <v>46190</v>
@@ -1088,7 +1094,7 @@
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B37" s="5">
         <v>46190</v>
@@ -1106,7 +1112,7 @@
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B38" s="5">
         <v>46191</v>
@@ -1124,7 +1130,7 @@
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B39" s="5">
         <v>46192</v>
@@ -1142,7 +1148,7 @@
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B40" s="5">
         <v>46192</v>
@@ -1160,7 +1166,7 @@
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B41" s="5">
         <v>46192</v>
@@ -1178,7 +1184,7 @@
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B42" s="5">
         <v>46193</v>
@@ -1192,7 +1198,7 @@
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B43" s="5">
         <v>46193</v>
@@ -1206,7 +1212,7 @@
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B44" s="5">
         <v>46194</v>
@@ -1220,7 +1226,7 @@
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B45" s="5">
         <v>46194</v>
@@ -1234,7 +1240,7 @@
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B46" s="5">
         <v>46196</v>
@@ -1248,7 +1254,7 @@
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B47" s="5">
         <v>46200</v>
@@ -1262,7 +1268,7 @@
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B48" s="5">
         <v>46200</v>
@@ -1276,7 +1282,7 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B49" s="5">
         <v>46201</v>
@@ -1290,7 +1296,7 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B50" s="10">
         <v>46202</v>
@@ -1304,7 +1310,7 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B51" s="10">
         <v>46203</v>
@@ -1318,7 +1324,7 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B52" s="10">
         <v>46203</v>
@@ -1332,7 +1338,7 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B53" s="10">
         <v>46203</v>
@@ -1346,7 +1352,7 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B54" s="10"/>
       <c r="C54" s="2"/>
@@ -1354,7 +1360,7 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" s="2">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -1362,7 +1368,7 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" s="2">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
@@ -1460,14 +1466,16 @@
       <c r="D5" s="4"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
+      <c r="A6" s="2">
+        <v>4</v>
+      </c>
       <c r="B6" s="5"/>
       <c r="C6" s="2"/>
       <c r="D6" s="4"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="2"/>
@@ -1475,7 +1483,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" s="5"/>
       <c r="C8" s="2"/>
@@ -1483,7 +1491,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="2"/>
@@ -1491,7 +1499,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="2"/>
@@ -1499,7 +1507,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="2"/>
@@ -1507,7 +1515,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="2"/>
@@ -1515,7 +1523,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="2"/>
@@ -1523,7 +1531,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B14" s="5"/>
       <c r="C14" s="2"/>
@@ -1531,7 +1539,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="2"/>
@@ -1539,7 +1547,7 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16" s="2"/>
@@ -1547,7 +1555,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="2"/>
@@ -1555,7 +1563,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="2"/>
@@ -1563,7 +1571,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="2"/>
@@ -1571,21 +1579,23 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="2"/>
       <c r="D20" s="4"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="2"/>
+      <c r="A21" s="2">
+        <v>19</v>
+      </c>
       <c r="B21" s="5"/>
       <c r="C21" s="2"/>
       <c r="D21" s="4"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="2"/>
@@ -1593,7 +1603,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="2"/>
@@ -1601,21 +1611,23 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B24" s="5"/>
       <c r="C24" s="2"/>
       <c r="D24" s="4"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="2"/>
+      <c r="A25" s="2">
+        <v>23</v>
+      </c>
       <c r="B25" s="5"/>
       <c r="C25" s="2"/>
       <c r="D25" s="4"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B26" s="5"/>
       <c r="C26" s="2"/>
@@ -1623,7 +1635,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="2"/>
@@ -1631,7 +1643,7 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="2"/>
@@ -1639,7 +1651,7 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B29" s="5"/>
       <c r="C29" s="2"/>
@@ -1647,7 +1659,7 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="2"/>
@@ -1655,7 +1667,7 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B31" s="5"/>
       <c r="C31" s="2"/>
@@ -1663,7 +1675,7 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="2"/>
@@ -1671,7 +1683,7 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B33" s="5"/>
       <c r="C33" s="2"/>
@@ -1679,7 +1691,7 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="2"/>
@@ -1687,7 +1699,7 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B35" s="5"/>
       <c r="C35" s="2"/>
@@ -1695,7 +1707,7 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B36" s="5"/>
       <c r="C36" s="2"/>
@@ -1703,7 +1715,7 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B37" s="5"/>
       <c r="C37" s="2"/>
@@ -1711,7 +1723,7 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B38" s="5"/>
       <c r="C38" s="2"/>
@@ -1719,7 +1731,7 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="2"/>
@@ -1727,7 +1739,7 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B40" s="5"/>
       <c r="C40" s="2"/>
@@ -1735,7 +1747,7 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B41" s="5"/>
       <c r="C41" s="2"/>
@@ -1743,7 +1755,7 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B42" s="5"/>
       <c r="C42" s="2"/>
@@ -1751,7 +1763,7 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B43" s="5"/>
       <c r="C43" s="2"/>
@@ -1759,7 +1771,7 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B44" s="5"/>
       <c r="C44" s="2"/>
@@ -1767,7 +1779,7 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B45" s="5"/>
       <c r="C45" s="2"/>
@@ -1775,7 +1787,7 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B46" s="5"/>
       <c r="C46" s="2"/>
@@ -1783,7 +1795,7 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B47" s="5"/>
       <c r="C47" s="2"/>
@@ -1791,7 +1803,7 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B48" s="5"/>
       <c r="C48" s="2"/>
@@ -1799,7 +1811,7 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B49" s="10"/>
       <c r="C49" s="2"/>
@@ -1807,7 +1819,7 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B50" s="10"/>
       <c r="C50" s="2"/>
@@ -1815,7 +1827,7 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B51" s="10"/>
       <c r="C51" s="2"/>
@@ -1823,32 +1835,26 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B52" s="10"/>
       <c r="C52" s="2"/>
       <c r="D52" s="4"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A53" s="2">
-        <v>48</v>
-      </c>
+      <c r="A53" s="2"/>
       <c r="B53" s="10"/>
       <c r="C53" s="2"/>
       <c r="D53" s="4"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A54" s="2">
-        <v>49</v>
-      </c>
+      <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
       <c r="D54" s="4"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A55" s="2">
-        <v>50</v>
-      </c>
+      <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
       <c r="D55" s="4"/>

</xml_diff>